<commit_message>
#651 Left steep slope collider
</commit_message>
<xml_diff>
--- a/Source/docs/edge collider points.xlsx
+++ b/Source/docs/edge collider points.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\SonicTheHedgehogFan\Source\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D144E7E-4A68-41F4-B629-C9709DD07388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF63E36-ADCD-4DA3-BFAE-63DA84E6CF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1035" yWindow="4185" windowWidth="10665" windowHeight="9945" tabRatio="294" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="294" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arcs" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
   <si>
     <t>X</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>Slope 2</t>
   </si>
 </sst>
 </file>
@@ -192,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -200,11 +203,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -968,7 +978,7 @@
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="7030A0"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -979,11 +989,11 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="7030A0"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:srgbClr val="7030A0"/>
+                  <a:schemeClr val="accent2"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
@@ -1047,6 +1057,412 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-E84B-4BC5-965B-998EFE63AC0E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="656837759"/>
+        <c:axId val="656832479"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="656837759"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="656832479"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="656832479"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="656837759"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>L1</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Slopes!$J$15:$J$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.36</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.75</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.15</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.75</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Slopes!$K$15:$K$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-049E-47C2-90B1-FF4C973EB2A4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>R1</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Slopes!$L$15:$L$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.35000000000000009</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.1399999999999997</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.9</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Slopes!$M$15:$M$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-049E-47C2-90B1-FF4C973EB2A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1310,6 +1726,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1827,6 +2283,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2392,13 +3364,13 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:rowOff>123826</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>161926</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2425,6 +3397,44 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>114301</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C3126D8-8C8E-44FF-847A-9FC58C2DE4B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2440,16 +3450,16 @@
     <tableColumn id="4" xr3:uid="{B4DA9531-DAA8-440F-A4F7-1651AEF7C9D0}" name="Y3">
       <calculatedColumnFormula>I4*-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{930412DB-E20E-4C7B-805D-500FF36DE3BC}" name="X4" dataDxfId="5">
+    <tableColumn id="5" xr3:uid="{930412DB-E20E-4C7B-805D-500FF36DE3BC}" name="X4" dataDxfId="7">
       <calculatedColumnFormula>Table1[[#This Row],[X]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{C51AFF9F-B38E-4E0C-B646-38CC0AD62AF1}" name="Y5" dataDxfId="4">
+    <tableColumn id="6" xr3:uid="{C51AFF9F-B38E-4E0C-B646-38CC0AD62AF1}" name="Y5" dataDxfId="6">
       <calculatedColumnFormula>Table1[[#This Row],[Y]]*-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F2DFE805-3168-4ADE-9BA5-29432CA43DB0}" name="X6" dataDxfId="3">
+    <tableColumn id="7" xr3:uid="{F2DFE805-3168-4ADE-9BA5-29432CA43DB0}" name="X6" dataDxfId="5">
       <calculatedColumnFormula>Table1[[#This Row],[Y]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4C1F46B4-FC82-48FE-967B-BB4B620F9340}" name="Y7" dataDxfId="2">
+    <tableColumn id="8" xr3:uid="{4C1F46B4-FC82-48FE-967B-BB4B620F9340}" name="Y7" dataDxfId="4">
       <calculatedColumnFormula>Table1[[#This Row],[X]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2464,11 +3474,29 @@
     <tableColumn id="1" xr3:uid="{365FA2AD-0A1E-4C5C-A2D8-54BCA54BF5DE}" name="n"/>
     <tableColumn id="5" xr3:uid="{69A97531-E11B-43D5-AD5D-570F4F494085}" name="X"/>
     <tableColumn id="2" xr3:uid="{E254CC5E-8892-4D40-99B6-622F493BEF38}" name="Y"/>
-    <tableColumn id="3" xr3:uid="{EB0823E3-57E4-4B80-8BB2-C463F15F2FC6}" name="X2" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{EB0823E3-57E4-4B80-8BB2-C463F15F2FC6}" name="X2" dataDxfId="3">
       <calculatedColumnFormula array="1">INDEX(Table2[X],MAX(Table2[n])-Table2[[#This Row],[n]]+1)*-1+MAX(Table2[X])-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{AAA31200-1775-4C5F-BB07-79082177C57E}" name="Y2" dataDxfId="1">
+    <tableColumn id="4" xr3:uid="{AAA31200-1775-4C5F-BB07-79082177C57E}" name="Y2" dataDxfId="2">
       <calculatedColumnFormula array="1">INDEX(Table2[Y],MAX(Table2[n])-Table2[[#This Row],[n]]+1)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{62E12B01-AFE2-482E-B396-92521B54F75F}" name="Table24" displayName="Table24" ref="I14:M22" totalsRowShown="0">
+  <autoFilter ref="I14:M22" xr:uid="{62E12B01-AFE2-482E-B396-92521B54F75F}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{DC063686-E555-4FAD-8221-EAAB386345AB}" name="n"/>
+    <tableColumn id="5" xr3:uid="{2BE63AD5-D0DA-4863-8F32-A3C9DAC74E3E}" name="X"/>
+    <tableColumn id="2" xr3:uid="{7B95F362-67D7-43EE-996D-1D7C17F604C4}" name="Y"/>
+    <tableColumn id="3" xr3:uid="{F72EF3AE-EC55-42AA-95EE-40A102D5B2D0}" name="X2" dataDxfId="1">
+      <calculatedColumnFormula array="1">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{0B5E9AAF-A05D-40DB-86C6-05E429311B97}" name="Y2" dataDxfId="0">
+      <calculatedColumnFormula array="1">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3076,7 +4104,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{305E9C1B-3DC9-48FB-B8F0-4E3C8835405B}">
-  <dimension ref="I1:M9"/>
+  <dimension ref="I1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="5.28515625" customWidth="1"/>
@@ -3226,12 +4254,198 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="J12" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I13" s="2"/>
+      <c r="J13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="2"/>
+      <c r="L13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M13" s="2"/>
+    </row>
+    <row r="14" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" t="s">
+        <v>0</v>
+      </c>
+      <c r="K14" t="s">
+        <v>1</v>
+      </c>
+      <c r="L14" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15" cm="1">
+        <f t="array" ref="L15">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>-1</v>
+      </c>
+      <c r="M15" cm="1">
+        <f t="array" ref="M15">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I16">
+        <v>2</v>
+      </c>
+      <c r="J16">
+        <v>0.6</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16" cm="1">
+        <f t="array" ref="L16">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>-0.25</v>
+      </c>
+      <c r="M16" cm="1">
+        <f t="array" ref="M16">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>0.17</v>
+      </c>
+      <c r="L17" cm="1">
+        <f t="array" ref="L17">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>0.35000000000000009</v>
+      </c>
+      <c r="M17" cm="1">
+        <f t="array" ref="M17">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="18" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I18">
+        <v>4</v>
+      </c>
+      <c r="J18">
+        <v>1.36</v>
+      </c>
+      <c r="K18">
+        <v>0.5</v>
+      </c>
+      <c r="L18" cm="1">
+        <f t="array" ref="L18">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>0.75</v>
+      </c>
+      <c r="M18" cm="1">
+        <f t="array" ref="M18">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="19" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I19">
+        <v>5</v>
+      </c>
+      <c r="J19">
+        <v>2.75</v>
+      </c>
+      <c r="K19">
+        <v>2.5</v>
+      </c>
+      <c r="L19" cm="1">
+        <f t="array" ref="L19">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>2.1399999999999997</v>
+      </c>
+      <c r="M19" cm="1">
+        <f t="array" ref="M19">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I20">
+        <v>6</v>
+      </c>
+      <c r="J20">
+        <v>3.15</v>
+      </c>
+      <c r="K20">
+        <v>2.8</v>
+      </c>
+      <c r="L20" cm="1">
+        <f t="array" ref="L20">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>2.5</v>
+      </c>
+      <c r="M20" cm="1">
+        <f t="array" ref="M20">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="21" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I21">
+        <v>7</v>
+      </c>
+      <c r="J21">
+        <v>3.75</v>
+      </c>
+      <c r="K21">
+        <v>3</v>
+      </c>
+      <c r="L21" s="7" cm="1">
+        <f t="array" ref="L21">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>2.9</v>
+      </c>
+      <c r="M21" s="7" cm="1">
+        <f t="array" ref="M21">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="9:13" x14ac:dyDescent="0.25">
+      <c r="I22">
+        <v>8</v>
+      </c>
+      <c r="J22">
+        <v>4.5</v>
+      </c>
+      <c r="K22">
+        <v>3</v>
+      </c>
+      <c r="L22" s="7" cm="1">
+        <f t="array" ref="L22">INDEX(Table24[X],MAX(Table24[n])-Table24[[#This Row],[n]]+1)*-1+MAX(Table24[X])-1</f>
+        <v>3.5</v>
+      </c>
+      <c r="M22" s="7" cm="1">
+        <f t="array" ref="M22">INDEX(Table24[Y],MAX(Table24[n])-Table24[[#This Row],[n]]+1)</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>